<commit_message>
4735 - remove wbs title from wbs report
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Tests/Resources/WbsBoeReport.xlsx
+++ b/GenBOE/GenBOE.Tests/Resources/WbsBoeReport.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="21929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9AADEA35-2D61-44D8-B5B2-4BDC99E54D47}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39327688-5AFA-489C-9A34-48189BF565BC}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="405" yWindow="1905" windowWidth="18900" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4080" yWindow="2730" windowWidth="18900" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WBS Summary of Hours, ODC Costs" sheetId="1" r:id="rId1"/>
@@ -15,15 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Total Hours</t>
   </si>
   <si>
     <t>WBS #</t>
-  </si>
-  <si>
-    <t>WBS Title</t>
   </si>
   <si>
     <t>Total Cost</t>
@@ -36,7 +33,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -58,8 +55,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF452DB2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,6 +100,36 @@
           <color theme="0" tint="-0.25098422193060094"/>
         </stop>
       </gradientFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF070729"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9F9F9F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF452DB2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD35714"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -97,11 +152,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -121,9 +182,15 @@
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="8">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="PPDuplicateRow" xfId="5" xr:uid="{8378614A-AC07-4B15-956E-22CDC7C40CFE}"/>
+    <cellStyle name="PPHeaderColumn" xfId="3" xr:uid="{D48D1087-32FE-4788-80EB-F9A38361FEC8}"/>
+    <cellStyle name="PPHeaderRequired" xfId="4" xr:uid="{687F2E1F-9313-4DA9-95AF-DABF90BA154F}"/>
+    <cellStyle name="PPHeaderTop" xfId="2" xr:uid="{D12BE062-B7F0-4E8B-8775-28E17ABA5827}"/>
+    <cellStyle name="PPInvalidValue" xfId="6" xr:uid="{88DC879F-97DF-400E-8318-C57E9EA893D5}"/>
+    <cellStyle name="PPMissingValue" xfId="7" xr:uid="{681BB475-C7AC-4315-BFA5-CAA8AF68FD2A}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -459,34 +526,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
-    <col min="2" max="3" width="25.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="25.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:4" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>